<commit_message>
Update questionIds in CN law & policy pages
</commit_message>
<xml_diff>
--- a/docs/总题库包含出现题库名.xlsx
+++ b/docs/总题库包含出现题库名.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hamwiki\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{557E85E0-4A31-4C08-9625-4261D2587BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6308E1DC-F8DC-4F9D-A00B-5363F9BD7C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24086,205 +24086,205 @@
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+      <c r="A81" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C81" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="D81" t="s">
+      <c r="D81" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="E81" t="s">
+      <c r="E81" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F81" t="s">
+      <c r="F81" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="G81" t="s">
+      <c r="G81" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="H81" t="s">
+      <c r="H81" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="I81" t="s">
+      <c r="I81" s="1" t="s">
         <v>448</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+      <c r="A82" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C82" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="D82" t="s">
+      <c r="D82" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="E82" t="s">
+      <c r="E82" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F82" t="s">
+      <c r="F82" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G82" t="s">
+      <c r="G82" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="H82" t="s">
+      <c r="H82" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="I82" t="s">
+      <c r="I82" s="1" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+      <c r="A83" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C83" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="D83" t="s">
+      <c r="D83" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="E83" t="s">
-        <v>9</v>
-      </c>
-      <c r="F83" t="s">
+      <c r="E83" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F83" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="G83" t="s">
+      <c r="G83" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="H83" t="s">
+      <c r="H83" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="I83" t="s">
+      <c r="I83" s="1" t="s">
         <v>460</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+      <c r="A84" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C84" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="D84" t="s">
+      <c r="D84" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="E84" t="s">
-        <v>9</v>
-      </c>
-      <c r="F84" t="s">
+      <c r="E84" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F84" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="G84" t="s">
+      <c r="G84" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="H84" t="s">
+      <c r="H84" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="I84" t="s">
+      <c r="I84" s="1" t="s">
         <v>466</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+      <c r="A85" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C85" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="D85" t="s">
+      <c r="D85" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="E85" t="s">
-        <v>9</v>
-      </c>
-      <c r="F85" t="s">
+      <c r="E85" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F85" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="G85" t="s">
+      <c r="G85" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="H85" t="s">
+      <c r="H85" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="I85" t="s">
+      <c r="I85" s="1" t="s">
         <v>472</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+      <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C86" t="s">
+      <c r="C86" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="D86" t="s">
+      <c r="D86" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="E86" t="s">
-        <v>5</v>
-      </c>
-      <c r="F86" t="s">
+      <c r="E86" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F86" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="G86" t="s">
+      <c r="G86" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="H86" t="s">
+      <c r="H86" s="1" t="s">
         <v>477</v>
       </c>
-      <c r="I86" t="s">
+      <c r="I86" s="1" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+      <c r="A87" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C87" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="D87" t="s">
+      <c r="D87" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="E87" t="s">
-        <v>5</v>
-      </c>
-      <c r="F87" t="s">
+      <c r="E87" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F87" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="G87" t="s">
+      <c r="G87" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="H87" t="s">
+      <c r="H87" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="I87" t="s">
+      <c r="I87" s="1" t="s">
         <v>484</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update question mappings and math quote block
Added new question IDs to the two law/policy wiki pages, fixed the final parallel-resistance formula block in `circuit-theory.md` so it stays within the quote formatting, and updated the corresponding question-bank spreadsheet source file.
</commit_message>
<xml_diff>
--- a/docs/总题库包含出现题库名.xlsx
+++ b/docs/总题库包含出现题库名.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hamwiki\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6308E1DC-F8DC-4F9D-A00B-5363F9BD7C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1FEBFB-2B80-4B1C-8A25-ED7FE725584A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24289,118 +24289,118 @@
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+      <c r="A88" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C88" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="D88" t="s">
+      <c r="D88" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="E88" t="s">
-        <v>9</v>
-      </c>
-      <c r="F88" t="s">
+      <c r="E88" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F88" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="G88" t="s">
+      <c r="G88" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="H88" t="s">
+      <c r="H88" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="I88" t="s">
+      <c r="I88" s="1" t="s">
         <v>490</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+      <c r="A89" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C89" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="D89" t="s">
+      <c r="D89" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="E89" t="s">
+      <c r="E89" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F89" t="s">
+      <c r="F89" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="G89" t="s">
+      <c r="G89" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="H89" t="s">
+      <c r="H89" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="I89" t="s">
+      <c r="I89" s="1" t="s">
         <v>496</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+      <c r="A90" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C90" s="1" t="s">
         <v>497</v>
       </c>
-      <c r="D90" t="s">
+      <c r="D90" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="E90" t="s">
-        <v>5</v>
-      </c>
-      <c r="F90" t="s">
+      <c r="E90" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F90" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="G90" t="s">
+      <c r="G90" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="H90" t="s">
+      <c r="H90" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="I90" t="s">
+      <c r="I90" s="1" t="s">
         <v>502</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+      <c r="A91" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C91" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="D91" t="s">
+      <c r="D91" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="E91" t="s">
-        <v>5</v>
-      </c>
-      <c r="F91" t="s">
+      <c r="E91" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F91" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="G91" t="s">
+      <c r="G91" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="H91" t="s">
+      <c r="H91" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="I91" t="s">
+      <c r="I91" s="1" t="s">
         <v>508</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add more callsign requirement question IDs
</commit_message>
<xml_diff>
--- a/docs/总题库包含出现题库名.xlsx
+++ b/docs/总题库包含出现题库名.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hamwiki\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1FEBFB-2B80-4B1C-8A25-ED7FE725584A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE19FE3-06B2-43D1-BEDB-F10C77EBED34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24405,292 +24405,292 @@
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>5</v>
-      </c>
-      <c r="B92" t="s">
+      <c r="A92" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B92" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C92" t="s">
+      <c r="C92" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="D92" t="s">
+      <c r="D92" s="1" t="s">
         <v>511</v>
       </c>
-      <c r="E92" t="s">
-        <v>5</v>
-      </c>
-      <c r="F92" t="s">
+      <c r="E92" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F92" s="1" t="s">
         <v>512</v>
       </c>
-      <c r="G92" t="s">
+      <c r="G92" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="H92" t="s">
+      <c r="H92" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="I92" t="s">
+      <c r="I92" s="1" t="s">
         <v>515</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>5</v>
-      </c>
-      <c r="B93" t="s">
+      <c r="A93" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B93" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C93" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="D93" t="s">
+      <c r="D93" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="E93" t="s">
-        <v>9</v>
-      </c>
-      <c r="F93" t="s">
+      <c r="E93" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F93" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="G93" t="s">
+      <c r="G93" s="1" t="s">
         <v>518</v>
       </c>
-      <c r="H93" t="s">
+      <c r="H93" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="I93" t="s">
+      <c r="I93" s="1" t="s">
         <v>520</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>5</v>
-      </c>
-      <c r="B94" t="s">
+      <c r="A94" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B94" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C94" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="D94" t="s">
+      <c r="D94" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="E94" t="s">
+      <c r="E94" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F94" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="G94" t="s">
+      <c r="G94" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="H94" t="s">
+      <c r="H94" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="I94" t="s">
+      <c r="I94" s="1" t="s">
         <v>525</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>5</v>
-      </c>
-      <c r="B95" t="s">
+      <c r="A95" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B95" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C95" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="D95" t="s">
+      <c r="D95" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="E95" t="s">
-        <v>9</v>
-      </c>
-      <c r="F95" t="s">
+      <c r="E95" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F95" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="G95" t="s">
+      <c r="G95" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="H95" t="s">
+      <c r="H95" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="I95" t="s">
+      <c r="I95" s="1" t="s">
         <v>530</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>5</v>
-      </c>
-      <c r="B96" t="s">
+      <c r="A96" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B96" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C96" t="s">
+      <c r="C96" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="D96" t="s">
+      <c r="D96" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="E96" t="s">
-        <v>9</v>
-      </c>
-      <c r="F96" t="s">
+      <c r="E96" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F96" s="1" t="s">
         <v>533</v>
       </c>
-      <c r="G96" t="s">
+      <c r="G96" s="1" t="s">
         <v>534</v>
       </c>
-      <c r="H96" t="s">
+      <c r="H96" s="1" t="s">
         <v>535</v>
       </c>
-      <c r="I96" t="s">
+      <c r="I96" s="1" t="s">
         <v>536</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>5</v>
-      </c>
-      <c r="B97" t="s">
+      <c r="A97" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B97" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C97" t="s">
+      <c r="C97" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D97" t="s">
+      <c r="D97" s="1" t="s">
         <v>538</v>
       </c>
-      <c r="E97" t="s">
-        <v>9</v>
-      </c>
-      <c r="F97" t="s">
+      <c r="E97" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F97" s="1" t="s">
         <v>539</v>
       </c>
-      <c r="G97" t="s">
+      <c r="G97" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="H97" t="s">
+      <c r="H97" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I97" t="s">
+      <c r="I97" s="1" t="s">
         <v>542</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>5</v>
-      </c>
-      <c r="B98" t="s">
+      <c r="A98" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B98" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C98" t="s">
+      <c r="C98" s="1" t="s">
         <v>543</v>
       </c>
-      <c r="D98" t="s">
+      <c r="D98" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="E98" t="s">
+      <c r="E98" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F98" t="s">
+      <c r="F98" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="G98" t="s">
+      <c r="G98" s="1" t="s">
         <v>520</v>
       </c>
-      <c r="H98" t="s">
+      <c r="H98" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="I98" t="s">
+      <c r="I98" s="1" t="s">
         <v>530</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>5</v>
-      </c>
-      <c r="B99" t="s">
+      <c r="A99" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B99" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C99" t="s">
+      <c r="C99" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="D99" t="s">
+      <c r="D99" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="E99" t="s">
+      <c r="E99" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F99" t="s">
+      <c r="F99" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="G99" t="s">
+      <c r="G99" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="H99" t="s">
+      <c r="H99" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="I99" t="s">
+      <c r="I99" s="1" t="s">
         <v>550</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>5</v>
-      </c>
-      <c r="B100" t="s">
+      <c r="A100" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B100" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C100" t="s">
+      <c r="C100" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="D100" t="s">
+      <c r="D100" s="1" t="s">
         <v>552</v>
       </c>
-      <c r="E100" t="s">
+      <c r="E100" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F100" t="s">
+      <c r="F100" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="G100" t="s">
+      <c r="G100" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="H100" t="s">
+      <c r="H100" s="1" t="s">
         <v>555</v>
       </c>
-      <c r="I100" t="s">
+      <c r="I100" s="1" t="s">
         <v>556</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>5</v>
-      </c>
-      <c r="B101" t="s">
+      <c r="A101" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B101" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C101" t="s">
+      <c r="C101" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="D101" t="s">
+      <c r="D101" s="1" t="s">
         <v>558</v>
       </c>
-      <c r="E101" t="s">
+      <c r="E101" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F101" t="s">
+      <c r="F101" s="1" t="s">
         <v>559</v>
       </c>
-      <c r="G101" t="s">
+      <c r="G101" s="1" t="s">
         <v>560</v>
       </c>
-      <c r="H101" t="s">
+      <c r="H101" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="I101" t="s">
+      <c r="I101" s="1" t="s">
         <v>548</v>
       </c>
     </row>

</xml_diff>